<commit_message>
docs: sync latest API specification workbook
</commit_message>
<xml_diff>
--- a/docs/BLOOM_MVP_API_명세서.xlsx
+++ b/docs/BLOOM_MVP_API_명세서.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="Rf6d847e9bd0c4a51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="엔드포인트" sheetId="2" r:id="R0456030045b44afd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request 필드" sheetId="3" r:id="R19c36bb7a0bc4ab0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response 필드" sheetId="4" r:id="R0038a6ea353940c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enum" sheetId="5" r:id="R61d0fdfeff16409b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="오류 코드" sheetId="6" r:id="R5645b3dba4e244b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="미확정" sheetId="7" r:id="R22ea4efd14074d25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 공개 API" sheetId="8" r:id="R43bd7593b4314905"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 내부 API" sheetId="9" r:id="R698aa52ce0ff4cdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 상태" sheetId="10" r:id="Ra7a5a401fc1f49a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="11" r:id="R7f01c8885272409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R34a99c5d639e4a2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="엔드포인트" sheetId="2" r:id="R7ce41bad6351459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request 필드" sheetId="3" r:id="Red91f4a09b674ecd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response 필드" sheetId="4" r:id="R11e697147d2f45fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enum" sheetId="5" r:id="Rbdeb3814676c4618"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="오류 코드" sheetId="6" r:id="Race09d2afb9e4443"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="미확정" sheetId="7" r:id="Rc2f87e313b004195"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 공개 API" sheetId="8" r:id="R53c2f9a5ad674c4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 내부 API" sheetId="9" r:id="Rcef8f9db9a624656"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 상태" sheetId="10" r:id="R4bd72ebdaaee4501"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="11" r:id="Rd39d34d135c846c3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -271,7 +271,7 @@
         <x:color rgb="FF137A3D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF7E7"/>
         </x:patternFill>
       </x:fill>
@@ -282,7 +282,7 @@
         <x:color rgb="FF9A6700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4E5"/>
         </x:patternFill>
       </x:fill>
@@ -293,7 +293,7 @@
         <x:color rgb="FF4338CA"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEEF2FF"/>
         </x:patternFill>
       </x:fill>
@@ -309,7 +309,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EndpointsTable" displayName="EndpointsTable" ref="A3:J31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EndpointsTable" displayName="EndpointsTable" ref="A3:J37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="도메인"/>
     <x:tableColumn id="2" name="Method"/>
@@ -327,7 +327,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequestFieldsTable" displayName="RequestFieldsTable" ref="A3:G43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RequestFieldsTable" displayName="RequestFieldsTable" ref="A3:G55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="DTO"/>
     <x:tableColumn id="2" name="필드명"/>
@@ -342,7 +342,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ResponseFieldsTable" displayName="ResponseFieldsTable" ref="A3:D45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ResponseFieldsTable" displayName="ResponseFieldsTable" ref="A3:D57" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="DTO"/>
     <x:tableColumn id="2" name="필드명"/>
@@ -391,7 +391,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AiPublicTable" displayName="AiPublicTable" ref="A3:I13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="AiPublicTable" displayName="AiPublicTable" ref="A3:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="도메인"/>
     <x:tableColumn id="2" name="Method"/>
@@ -715,8 +715,7 @@
         <x:v>전체 엔드포인트</x:v>
       </x:c>
       <x:c r="E5" s="10" t="n">
-        <x:f>COUNTA('엔드포인트'!$C$4:$C$200)</x:f>
-        <x:v>28</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -745,8 +744,7 @@
         <x:v>예정</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:f>COUNTIF('엔드포인트'!$I$4:$I$200,"예정")</x:f>
-        <x:v>3</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -767,7 +765,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="24" t="str">
-        <x:v>현재 구현 기준: 인증·온보딩·프로필·일일 기록·식단·활동·눈바디 사진 CRUD. AI 식단·예상 이미지·추천 시술은 예정입니다.</x:v>
+        <x:v>현재 구현 기준: 인증·온보딩·프로필·일일 기록·식단·활동·눈바디 사진 CRUD. AI 식단 계약은 확정됐으며 실제 AI 호출·예상 이미지·추천 시술은 구현 예정입니다.</x:v>
       </x:c>
       <x:c r="B12" s="24"/>
       <x:c r="C12" s="24"/>
@@ -824,7 +822,7 @@
         <x:v>식단</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>foodName/kcal/carbs/protein/fat 사용</x:v>
+        <x:v>foodName/kcal/carbs/protein/fat 사용, 미상 영양소는 null</x:v>
       </x:c>
       <x:c r="C17" s="28" t="str"/>
       <x:c r="D17" s="28" t="str"/>
@@ -943,10 +941,10 @@
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="38" t="str">
-        <x:v>CONFIRMED</x:v>
+        <x:v>RECORDED</x:v>
       </x:c>
       <x:c r="B6" s="33" t="str">
-        <x:v>사용자 수정·확정 완료</x:v>
+        <x:v>기록하기로 일반 식단 저장 완료</x:v>
       </x:c>
       <x:c r="C6" s="33" t="str">
         <x:v>일일 합계 반영</x:v>
@@ -1027,7 +1025,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f7e8ab8410640b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22d0af9ca7a54b2e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2056,28 +2054,28 @@
         <x:v>POST</x:v>
       </x:c>
       <x:c r="C29" s="33" t="str">
-        <x:v>/api/v1/ai/nutrition</x:v>
+        <x:v>/api/v1/ai/nutrition/analyses</x:v>
       </x:c>
       <x:c r="D29" s="33" t="str">
-        <x:v>사진/텍스트 영양 분석</x:v>
+        <x:v>사진 또는 텍스트 영양 분석</x:v>
       </x:c>
       <x:c r="E29" s="33" t="str">
         <x:v>필요</x:v>
       </x:c>
       <x:c r="F29" s="33" t="str">
-        <x:v>미확정</x:v>
+        <x:v>multipart: date,mealType,inputType,image|text</x:v>
       </x:c>
       <x:c r="G29" s="33" t="str">
-        <x:v>미확정</x:v>
+        <x:v>NutritionAnalysisResponse</x:v>
       </x:c>
       <x:c r="H29" s="33" t="str">
-        <x:v>-</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="I29" s="33" t="str">
-        <x:v>예정</x:v>
+        <x:v>명세 확정</x:v>
       </x:c>
       <x:c r="J29" s="33" t="str">
-        <x:v>DRAFT→수정→확정</x:v>
+        <x:v>IMAGE/TEXT 동시 전송 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="28" customHeight="1">
@@ -2142,6 +2140,196 @@
       </x:c>
       <x:c r="J31" s="33" t="str">
         <x:v>병원 예약·결제 제외</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>분석 상태·초안 조회</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>Path: analysisId</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>NutritionAnalysisResponse</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I32" t="str">
+        <x:v>명세 확정</x:v>
+      </x:c>
+      <x:c r="J32" t="str">
+        <x:v>PROCESSING/DRAFT/FAILED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>초안 음식 직접 추가</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="I33" t="str">
+        <x:v>명세 확정</x:v>
+      </x:c>
+      <x:c r="J33" t="str">
+        <x:v>source=USER_INPUT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>PATCH</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>초안 음식 수정</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I34" t="str">
+        <x:v>명세 확정</x:v>
+      </x:c>
+      <x:c r="J34" t="str">
+        <x:v>음식명·양·kcal·탄단지 수정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>DELETE</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>초안 음식 삭제</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="H35" t="str">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="I35" t="str">
+        <x:v>명세 확정</x:v>
+      </x:c>
+      <x:c r="J35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/record</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>초안을 일반 식단으로 기록</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>Path: analysisId</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>MealResponse[]</x:v>
+      </x:c>
+      <x:c r="H36" t="str">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="I36" t="str">
+        <x:v>명세 확정</x:v>
+      </x:c>
+      <x:c r="J36" t="str">
+        <x:v>별도 확정 단계 없음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>DELETE</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>분석 초안 취소</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="H37" t="str">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="I37" t="str">
+        <x:v>명세 확정</x:v>
+      </x:c>
+      <x:c r="J37" t="str">
+        <x:v>DRAFT는 7일 후 자동 삭제</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2155,7 +2343,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dea1831c9cc4648"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05e6edcc6e754597"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2894,13 +3082,13 @@
         <x:v>kcal</x:v>
       </x:c>
       <x:c r="C32" s="33" t="str">
-        <x:v>integer</x:v>
+        <x:v>integer|null</x:v>
       </x:c>
       <x:c r="D32" s="33" t="str">
-        <x:v>O</x:v>
+        <x:v>X</x:v>
       </x:c>
       <x:c r="E32" s="33" t="str">
-        <x:v>0~10000</x:v>
+        <x:v>0~10000; 미상=null</x:v>
       </x:c>
       <x:c r="F32" s="33" t="str">
         <x:v>320</x:v>
@@ -2917,13 +3105,13 @@
         <x:v>carbs</x:v>
       </x:c>
       <x:c r="C33" s="33" t="str">
-        <x:v>integer</x:v>
+        <x:v>integer|null</x:v>
       </x:c>
       <x:c r="D33" s="33" t="str">
-        <x:v>O</x:v>
+        <x:v>X</x:v>
       </x:c>
       <x:c r="E33" s="33" t="str">
-        <x:v>0~1000g</x:v>
+        <x:v>0~1000g; 미상=null</x:v>
       </x:c>
       <x:c r="F33" s="33" t="str">
         <x:v>60</x:v>
@@ -2940,13 +3128,13 @@
         <x:v>protein</x:v>
       </x:c>
       <x:c r="C34" s="33" t="str">
-        <x:v>integer</x:v>
+        <x:v>integer|null</x:v>
       </x:c>
       <x:c r="D34" s="33" t="str">
-        <x:v>O</x:v>
+        <x:v>X</x:v>
       </x:c>
       <x:c r="E34" s="33" t="str">
-        <x:v>0~1000g</x:v>
+        <x:v>0~1000g; 미상=null</x:v>
       </x:c>
       <x:c r="F34" s="33" t="str">
         <x:v>8</x:v>
@@ -2963,13 +3151,13 @@
         <x:v>fat</x:v>
       </x:c>
       <x:c r="C35" s="33" t="str">
-        <x:v>integer</x:v>
+        <x:v>integer|null</x:v>
       </x:c>
       <x:c r="D35" s="33" t="str">
-        <x:v>O</x:v>
+        <x:v>X</x:v>
       </x:c>
       <x:c r="E35" s="33" t="str">
-        <x:v>0~1000g</x:v>
+        <x:v>0~1000g; 미상=null</x:v>
       </x:c>
       <x:c r="F35" s="33" t="str">
         <x:v>3</x:v>
@@ -3160,6 +3348,282 @@
       </x:c>
       <x:c r="G43" s="33" t="str">
         <x:v>눈바디</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>NutritionAnalysisRequest</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>기록일</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>2026-08-16</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>NutritionAnalysisRequest</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>mealType</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>BREAKFAST/LUNCH/DINNER/SNACK</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>LUNCH</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>NutritionAnalysisRequest</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>inputType</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>IMAGE 또는 TEXT</x:v>
+      </x:c>
+      <x:c r="F46" t="str">
+        <x:v>IMAGE</x:v>
+      </x:c>
+      <x:c r="G46" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>NutritionAnalysisRequest</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>image</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>file</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>조건부</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>IMAGE일 때 필수; JPEG/PNG/WebP; 최대 10MB</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:v>meal.jpg</x:v>
+      </x:c>
+      <x:c r="G47" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>NutritionAnalysisRequest</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>조건부</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>TEXT일 때 필수; image와 동시 전송 불가</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>현미밥과 닭가슴살</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>foodName</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>최대 100자</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>현미밥</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>amount</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>decimal</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>0 이상</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>amountUnit</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>g/ml/serving 등</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="G51" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>kcal</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>미상=null</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="G52" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>carbs</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>미상=null</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G53" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>protein</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>미상=null</x:v>
+      </x:c>
+      <x:c r="F54" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G54" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>fat</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>미상=null</x:v>
+      </x:c>
+      <x:c r="F55" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G55" t="str">
+        <x:v>AI 식단</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3168,7 +3632,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd366bda741f1459d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e06c40a28bc47cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3331,7 +3795,7 @@
         <x:v>skin</x:v>
       </x:c>
       <x:c r="C11" s="33" t="str">
-        <x:v>string[]</x:v>
+        <x:v>SkinTag[]</x:v>
       </x:c>
       <x:c r="D11" s="33" t="str">
         <x:v>피부 태그</x:v>
@@ -3597,10 +4061,10 @@
         <x:v>kcal</x:v>
       </x:c>
       <x:c r="C30" s="33" t="str">
-        <x:v>integer</x:v>
+        <x:v>integer|null</x:v>
       </x:c>
       <x:c r="D30" s="33" t="str">
-        <x:v>칼로리</x:v>
+        <x:v>칼로리; 미상=null</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
@@ -3611,10 +4075,10 @@
         <x:v>carbs</x:v>
       </x:c>
       <x:c r="C31" s="33" t="str">
-        <x:v>integer</x:v>
+        <x:v>integer|null</x:v>
       </x:c>
       <x:c r="D31" s="33" t="str">
-        <x:v>탄수화물 g</x:v>
+        <x:v>탄수화물 g; 미상=null</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28" customHeight="1">
@@ -3625,10 +4089,10 @@
         <x:v>protein</x:v>
       </x:c>
       <x:c r="C32" s="33" t="str">
-        <x:v>integer</x:v>
+        <x:v>integer|null</x:v>
       </x:c>
       <x:c r="D32" s="33" t="str">
-        <x:v>단백질 g</x:v>
+        <x:v>단백질 g; 미상=null</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
@@ -3639,10 +4103,10 @@
         <x:v>fat</x:v>
       </x:c>
       <x:c r="C33" s="33" t="str">
-        <x:v>integer</x:v>
+        <x:v>integer|null</x:v>
       </x:c>
       <x:c r="D33" s="33" t="str">
-        <x:v>지방 g</x:v>
+        <x:v>지방 g; 미상=null</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
@@ -3811,6 +4275,174 @@
       </x:c>
       <x:c r="D45" s="33" t="str">
         <x:v>수정 시각</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>DailyDiaryResponse</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>nutritionIncomplete</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>하나 이상의 식단 영양정보가 null인지 여부</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>NutritionAnalysisResponse</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>analysisId</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>long</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>AI 분석 ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>NutritionAnalysisResponse</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>PROCESSING/DRAFT/RECORDED/FAILED/CANCELLED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>NutritionAnalysisResponse</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>modelVersion</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>분석 모델·버전</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>NutritionAnalysisResponse</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>foods</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>DraftFoodResponse[]</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>한 사진에서 인식한 여러 음식</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>NutritionAnalysisResponse</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>totalKcal</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>확인 가능한 kcal 합계</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>NutritionAnalysisResponse</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>manualInputAvailable</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>boolean</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>실패 시 직접 입력 가능 여부</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>draftFoodId</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>long</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>초안 음식 ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>amount</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>decimal|null</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>추정·수정 가능한 음식 양</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>amountUnit</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>string|null</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>음식 양 단위</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>source</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>MFDS/AI_ESTIMATE/USER_INPUT/USER_CORRECTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>confidence</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>decimal|null</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>내부 신뢰도; 사용자에게 숫자 미표시</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3819,7 +4451,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3688b03f3e0f488b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R620389ad3b9d4741"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4568,7 +5200,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf538b70a8b024d50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf914ba74e6484577"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4827,7 +5459,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f911b0f30d24030"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c115b038bad43d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5002,7 +5634,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69bb21d406954598"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cbe20c5d2564321"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5126,16 +5758,16 @@
         <x:v>multipart</x:v>
       </x:c>
       <x:c r="F4" s="33" t="str">
-        <x:v>date, mealType, image?, text?</x:v>
+        <x:v>date,mealType,inputType,image 또는 text</x:v>
       </x:c>
       <x:c r="G4" s="33" t="str">
         <x:v>NutritionAnalysisResponse</x:v>
       </x:c>
       <x:c r="H4" s="33" t="str">
-        <x:v>DRAFT</x:v>
+        <x:v>PROCESSING/DRAFT</x:v>
       </x:c>
       <x:c r="I4" s="33" t="str">
-        <x:v>초안</x:v>
+        <x:v>확정</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
@@ -5164,7 +5796,7 @@
         <x:v>PROCESSING/DRAFT/FAILED</x:v>
       </x:c>
       <x:c r="I5" s="33" t="str">
-        <x:v>초안</x:v>
+        <x:v>확정</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
@@ -5178,13 +5810,13 @@
         <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
-        <x:v>AI 추론 음식 사용자 수정</x:v>
+        <x:v>AI 초안 음식 사용자 수정</x:v>
       </x:c>
       <x:c r="E6" s="33" t="str">
         <x:v>JSON</x:v>
       </x:c>
       <x:c r="F6" s="33" t="str">
-        <x:v>foodName,kcal,carbs,protein,fat</x:v>
+        <x:v>foodName,amount,amountUnit,kcal,carbs,protein,fat</x:v>
       </x:c>
       <x:c r="G6" s="33" t="str">
         <x:v>DraftFoodResponse</x:v>
@@ -5193,7 +5825,7 @@
         <x:v>DRAFT</x:v>
       </x:c>
       <x:c r="I6" s="33" t="str">
-        <x:v>초안</x:v>
+        <x:v>확정</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -5204,10 +5836,10 @@
         <x:v>POST</x:v>
       </x:c>
       <x:c r="C7" s="33" t="str">
-        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/confirm</x:v>
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/record</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
-        <x:v>수정 결과를 일반 식단으로 확정</x:v>
+        <x:v>수정 여부와 관계없이 일반 식단으로 기록</x:v>
       </x:c>
       <x:c r="E7" s="33" t="str">
         <x:v>-</x:v>
@@ -5219,10 +5851,10 @@
         <x:v>MealResponse[]</x:v>
       </x:c>
       <x:c r="H7" s="33" t="str">
-        <x:v>CONFIRMED</x:v>
+        <x:v>RECORDED</x:v>
       </x:c>
       <x:c r="I7" s="33" t="str">
-        <x:v>초안</x:v>
+        <x:v>확정</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
@@ -5251,7 +5883,7 @@
         <x:v>CANCELLED</x:v>
       </x:c>
       <x:c r="I8" s="33" t="str">
-        <x:v>초안</x:v>
+        <x:v>확정</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
@@ -5397,6 +6029,64 @@
       </x:c>
       <x:c r="I13" s="33" t="str">
         <x:v>초안</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>초안 음식 직접 추가</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>JSON</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>DRAFT</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>DELETE</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>초안 음식 삭제</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>Path: analysisId,draftFoodId</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>DRAFT</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>확정</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5405,7 +6095,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1813044b713f470d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1941aada9a214b10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5568,7 +6258,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf33b61accd8d46a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae152ef940f24c0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add meal recommendations and fix mileage locking
</commit_message>
<xml_diff>
--- a/docs/BLOOM_MVP_API_명세서.xlsx
+++ b/docs/BLOOM_MVP_API_명세서.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R34a99c5d639e4a2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="엔드포인트" sheetId="2" r:id="R7ce41bad6351459b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request 필드" sheetId="3" r:id="Red91f4a09b674ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response 필드" sheetId="4" r:id="R11e697147d2f45fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enum" sheetId="5" r:id="Rbdeb3814676c4618"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="오류 코드" sheetId="6" r:id="Race09d2afb9e4443"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="미확정" sheetId="7" r:id="Rc2f87e313b004195"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 공개 API" sheetId="8" r:id="R53c2f9a5ad674c4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 내부 API" sheetId="9" r:id="Rcef8f9db9a624656"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 상태" sheetId="10" r:id="R4bd72ebdaaee4501"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="11" r:id="Rd39d34d135c846c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R1bb7d3da78bc4e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="엔드포인트" sheetId="2" r:id="Rd101f88718f74761"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request 필드" sheetId="3" r:id="R242aee1104204d80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response 필드" sheetId="4" r:id="R21e2ac9c879e4887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enum" sheetId="5" r:id="R3ee670073fa544c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="오류 코드" sheetId="6" r:id="R9cb844dff58f4fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="미확정" sheetId="7" r:id="Re48dc80bd5b44967"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 공개 API" sheetId="8" r:id="R112e99a38d7a4747"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 내부 API" sheetId="9" r:id="R0781a1c4c79c4463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI 상태" sheetId="10" r:id="Rfc6eb573436e48d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="11" r:id="R2d5b5902b56d4f76"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="17">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -83,8 +83,46 @@
       <x:color rgb="FF137A3D"/>
       <x:name val="Consolas"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF263244"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF263244"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF087A3D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF263244"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF087A3D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF2FC674"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF2FC674"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -116,8 +154,23 @@
         <x:fgColor rgb="FFFFF4E5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F8ED"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC8F1D3"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="15">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -174,11 +227,65 @@
         <x:color rgb="FFD9E1E7"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7E3DA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1E7"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E1E7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7E3DA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7E3DA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1E7"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E1E7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7E3DA"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD9E1E7"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E1E7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7E3DA"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7E3DA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD7E3DA"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7E3DA"/>
+      </x:left>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="41">
+  <x:cellXfs count="91">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -258,6 +365,136 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="9" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="8" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -695,7 +932,7 @@
         <x:v>기준 버전</x:v>
       </x:c>
       <x:c r="B4" s="8" t="str">
-        <x:v>2026-08-16</x:v>
+        <x:v>2026-08-19</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
         <x:v>지표</x:v>
@@ -715,7 +952,7 @@
         <x:v>전체 엔드포인트</x:v>
       </x:c>
       <x:c r="E5" s="10" t="n">
-        <x:v>34</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -729,8 +966,7 @@
         <x:v>완료</x:v>
       </x:c>
       <x:c r="E6" s="10" t="n">
-        <x:f>COUNTIF('엔드포인트'!$I$4:$I$200,"완료")</x:f>
-        <x:v>21</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -744,7 +980,7 @@
         <x:v>예정</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -765,7 +1001,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="24" t="str">
-        <x:v>현재 구현 기준: 인증·온보딩·프로필·일일 기록·식단·활동·눈바디 사진 CRUD. AI 식단 계약은 확정됐으며 실제 AI 호출·예상 이미지·추천 시술은 구현 예정입니다.</x:v>
+        <x:v>현재 구현 기준: 인증·프로필·일일·생리 기록·식단·활동·눈바디·업로드·마일리지 CRUD와 AI 채팅·식단 분석·추천 식단·추천 시술·기간 리포트를 구현했습니다. 눈바디 예상 이미지만 후순위입니다.</x:v>
       </x:c>
       <x:c r="B12" s="24"/>
       <x:c r="C12" s="24"/>
@@ -1025,7 +1261,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22d0af9ca7a54b2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2a21f6ccdc24f34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2072,7 +2308,7 @@
         <x:v>202</x:v>
       </x:c>
       <x:c r="I29" s="33" t="str">
-        <x:v>명세 확정</x:v>
+        <x:v>완료</x:v>
       </x:c>
       <x:c r="J29" s="33" t="str">
         <x:v>IMAGE/TEXT 동시 전송 불가</x:v>
@@ -2110,226 +2346,766 @@
         <x:v>AI 후순위</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="28" customHeight="1">
-      <x:c r="A31" s="33" t="str">
+    <x:row r="31" ht="30" customHeight="1">
+      <x:c r="A31" s="45" t="str">
         <x:v>추천 시술</x:v>
       </x:c>
-      <x:c r="B31" s="37" t="str">
+      <x:c r="B31" s="75" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C31" s="47" t="str">
+        <x:v>/api/v1/ai/procedures/recommendations</x:v>
+      </x:c>
+      <x:c r="D31" s="47" t="str">
+        <x:v>눈바디 기반 시술 추천</x:v>
+      </x:c>
+      <x:c r="E31" s="47" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F31" s="47" t="str">
+        <x:v>ProcedureRecommendationRequest</x:v>
+      </x:c>
+      <x:c r="G31" s="47" t="str">
+        <x:v>ProcedureRecommendationsResponse</x:v>
+      </x:c>
+      <x:c r="H31" s="47" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I31" s="50" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J31" s="48" t="str">
+        <x:v>bodyCheckId만 전송</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="30" customHeight="1">
+      <x:c r="A32" s="59" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B32" s="76" t="str">
         <x:v>GET</x:v>
       </x:c>
-      <x:c r="C31" s="33" t="str">
-        <x:v>/api/v1/procedures/recommendations</x:v>
-      </x:c>
-      <x:c r="D31" s="33" t="str">
-        <x:v>추천 시술 조회</x:v>
-      </x:c>
-      <x:c r="E31" s="33" t="str">
+      <x:c r="C32" s="60" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}</x:v>
+      </x:c>
+      <x:c r="D32" s="60" t="str">
+        <x:v>분석 상태·초안 조회</x:v>
+      </x:c>
+      <x:c r="E32" s="60" t="str">
         <x:v>필요</x:v>
       </x:c>
-      <x:c r="F31" s="33" t="str">
-        <x:v>미확정</x:v>
-      </x:c>
-      <x:c r="G31" s="33" t="str">
-        <x:v>미확정</x:v>
-      </x:c>
-      <x:c r="H31" s="33" t="str">
+      <x:c r="F32" s="60" t="str">
+        <x:v>Path: analysisId</x:v>
+      </x:c>
+      <x:c r="G32" s="60" t="str">
+        <x:v>NutritionAnalysisResponse</x:v>
+      </x:c>
+      <x:c r="H32" s="60" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I32" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J32" s="61" t="str">
+        <x:v>PROCESSING/DRAFT/FAILED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="30" customHeight="1">
+      <x:c r="A33" s="72" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B33" s="77" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C33" s="73" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods</x:v>
+      </x:c>
+      <x:c r="D33" s="73" t="str">
+        <x:v>초안 음식 직접 추가</x:v>
+      </x:c>
+      <x:c r="E33" s="73" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F33" s="73" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="G33" s="73" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="H33" s="73" t="str">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="I33" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J33" s="74" t="str">
+        <x:v>source=USER_INPUT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="30" customHeight="1">
+      <x:c r="A34" s="59" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B34" s="76" t="str">
+        <x:v>PATCH</x:v>
+      </x:c>
+      <x:c r="C34" s="60" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
+      </x:c>
+      <x:c r="D34" s="60" t="str">
+        <x:v>초안 음식 수정</x:v>
+      </x:c>
+      <x:c r="E34" s="60" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F34" s="60" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="G34" s="60" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="H34" s="60" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I34" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J34" s="61" t="str">
+        <x:v>음식명·양·kcal·탄단지 수정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="30" customHeight="1">
+      <x:c r="A35" s="72" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B35" s="77" t="str">
+        <x:v>DELETE</x:v>
+      </x:c>
+      <x:c r="C35" s="73" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
+      </x:c>
+      <x:c r="D35" s="73" t="str">
+        <x:v>초안 음식 삭제</x:v>
+      </x:c>
+      <x:c r="E35" s="73" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F35" s="73" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="I31" s="33" t="str">
-        <x:v>예정</x:v>
-      </x:c>
-      <x:c r="J31" s="33" t="str">
-        <x:v>병원 예약·결제 제외</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" t="str">
+      <x:c r="G35" s="73" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="H35" s="73" t="str">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="I35" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J35" s="74"/>
+    </x:row>
+    <x:row r="36" ht="30" customHeight="1">
+      <x:c r="A36" s="59" t="str">
         <x:v>AI 식단</x:v>
       </x:c>
-      <x:c r="B32" t="str">
+      <x:c r="B36" s="76" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C36" s="60" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/record</x:v>
+      </x:c>
+      <x:c r="D36" s="60" t="str">
+        <x:v>초안을 일반 식단으로 기록</x:v>
+      </x:c>
+      <x:c r="E36" s="60" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F36" s="60" t="str">
+        <x:v>Path: analysisId</x:v>
+      </x:c>
+      <x:c r="G36" s="60" t="str">
+        <x:v>MealResponse[]</x:v>
+      </x:c>
+      <x:c r="H36" s="60" t="str">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="I36" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J36" s="61" t="str">
+        <x:v>별도 확정 단계 없음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="30" customHeight="1">
+      <x:c r="A37" s="72" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B37" s="77" t="str">
+        <x:v>DELETE</x:v>
+      </x:c>
+      <x:c r="C37" s="73" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}</x:v>
+      </x:c>
+      <x:c r="D37" s="73" t="str">
+        <x:v>분석 초안 취소</x:v>
+      </x:c>
+      <x:c r="E37" s="73" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F37" s="73" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G37" s="73" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="H37" s="73" t="str">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="I37" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J37" s="74" t="str">
+        <x:v>DRAFT는 7일 후 자동 삭제</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="A38" s="59" t="str">
+        <x:v>업로드</x:v>
+      </x:c>
+      <x:c r="B38" s="76" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C38" s="60" t="str">
+        <x:v>/api/v1/uploads/images</x:v>
+      </x:c>
+      <x:c r="D38" s="60" t="str">
+        <x:v>인증 이미지 업로드</x:v>
+      </x:c>
+      <x:c r="E38" s="60" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F38" s="60" t="str">
+        <x:v>multipart: file,purpose</x:v>
+      </x:c>
+      <x:c r="G38" s="60" t="str">
+        <x:v>ImageUploadResponse</x:v>
+      </x:c>
+      <x:c r="H38" s="60" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="I38" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J38" s="61" t="str">
+        <x:v>JPEG/PNG/WebP, 최대 10MB</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="30" customHeight="1">
+      <x:c r="A39" s="72" t="str">
+        <x:v>업로드</x:v>
+      </x:c>
+      <x:c r="B39" s="77" t="str">
         <x:v>GET</x:v>
       </x:c>
-      <x:c r="C32" t="str">
-        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}</x:v>
-      </x:c>
-      <x:c r="D32" t="str">
-        <x:v>분석 상태·초안 조회</x:v>
-      </x:c>
-      <x:c r="E32" t="str">
+      <x:c r="C39" s="73" t="str">
+        <x:v>/api/v1/uploads/images/{imageId}</x:v>
+      </x:c>
+      <x:c r="D39" s="73" t="str">
+        <x:v>인증 이미지 조회</x:v>
+      </x:c>
+      <x:c r="E39" s="73" t="str">
         <x:v>필요</x:v>
       </x:c>
-      <x:c r="F32" t="str">
-        <x:v>Path: analysisId</x:v>
-      </x:c>
-      <x:c r="G32" t="str">
-        <x:v>NutritionAnalysisResponse</x:v>
-      </x:c>
-      <x:c r="H32" t="str">
+      <x:c r="F39" s="73" t="str">
+        <x:v>Path: imageId</x:v>
+      </x:c>
+      <x:c r="G39" s="73" t="str">
+        <x:v>binary image</x:v>
+      </x:c>
+      <x:c r="H39" s="73" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="I32" t="str">
-        <x:v>명세 확정</x:v>
-      </x:c>
-      <x:c r="J32" t="str">
-        <x:v>PROCESSING/DRAFT/FAILED</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" t="str">
-        <x:v>AI 식단</x:v>
-      </x:c>
-      <x:c r="B33" t="str">
+      <x:c r="I39" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J39" s="74" t="str">
+        <x:v>소유 사용자만 접근</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="30" customHeight="1">
+      <x:c r="A40" s="59" t="str">
+        <x:v>생리 기록</x:v>
+      </x:c>
+      <x:c r="B40" s="76" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="C33" t="str">
-        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods</x:v>
-      </x:c>
-      <x:c r="D33" t="str">
-        <x:v>초안 음식 직접 추가</x:v>
-      </x:c>
-      <x:c r="E33" t="str">
+      <x:c r="C40" s="60" t="str">
+        <x:v>/api/v1/periods</x:v>
+      </x:c>
+      <x:c r="D40" s="60" t="str">
+        <x:v>생리 기간 생성</x:v>
+      </x:c>
+      <x:c r="E40" s="60" t="str">
         <x:v>필요</x:v>
       </x:c>
-      <x:c r="F33" t="str">
-        <x:v>DraftFoodRequest</x:v>
-      </x:c>
-      <x:c r="G33" t="str">
-        <x:v>DraftFoodResponse</x:v>
-      </x:c>
-      <x:c r="H33" t="str">
+      <x:c r="F40" s="60" t="str">
+        <x:v>PeriodCreateRequest</x:v>
+      </x:c>
+      <x:c r="G40" s="60" t="str">
+        <x:v>PeriodResponse</x:v>
+      </x:c>
+      <x:c r="H40" s="60" t="n">
         <x:v>201</x:v>
       </x:c>
-      <x:c r="I33" t="str">
-        <x:v>명세 확정</x:v>
-      </x:c>
-      <x:c r="J33" t="str">
-        <x:v>source=USER_INPUT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" t="str">
-        <x:v>AI 식단</x:v>
-      </x:c>
-      <x:c r="B34" t="str">
+      <x:c r="I40" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J40" s="61" t="str">
+        <x:v>startDate &lt;= endDate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="30" customHeight="1">
+      <x:c r="A41" s="72" t="str">
+        <x:v>생리 기록</x:v>
+      </x:c>
+      <x:c r="B41" s="77" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C41" s="73" t="str">
+        <x:v>/api/v1/periods</x:v>
+      </x:c>
+      <x:c r="D41" s="73" t="str">
+        <x:v>생리 기간 목록</x:v>
+      </x:c>
+      <x:c r="E41" s="73" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F41" s="73" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G41" s="73" t="str">
+        <x:v>PeriodResponse[]</x:v>
+      </x:c>
+      <x:c r="H41" s="73" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I41" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J41" s="74" t="str">
+        <x:v>시작일 최신순</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="30" customHeight="1">
+      <x:c r="A42" s="59" t="str">
+        <x:v>생리 기록</x:v>
+      </x:c>
+      <x:c r="B42" s="76" t="str">
         <x:v>PATCH</x:v>
       </x:c>
-      <x:c r="C34" t="str">
-        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
-      </x:c>
-      <x:c r="D34" t="str">
-        <x:v>초안 음식 수정</x:v>
-      </x:c>
-      <x:c r="E34" t="str">
+      <x:c r="C42" s="60" t="str">
+        <x:v>/api/v1/periods/{periodId}</x:v>
+      </x:c>
+      <x:c r="D42" s="60" t="str">
+        <x:v>생리 기간 부분 수정</x:v>
+      </x:c>
+      <x:c r="E42" s="60" t="str">
         <x:v>필요</x:v>
       </x:c>
-      <x:c r="F34" t="str">
-        <x:v>DraftFoodRequest</x:v>
-      </x:c>
-      <x:c r="G34" t="str">
-        <x:v>DraftFoodResponse</x:v>
-      </x:c>
-      <x:c r="H34" t="str">
+      <x:c r="F42" s="60" t="str">
+        <x:v>PeriodPatchRequest</x:v>
+      </x:c>
+      <x:c r="G42" s="60" t="str">
+        <x:v>PeriodResponse</x:v>
+      </x:c>
+      <x:c r="H42" s="60" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="I34" t="str">
-        <x:v>명세 확정</x:v>
-      </x:c>
-      <x:c r="J34" t="str">
-        <x:v>음식명·양·kcal·탄단지 수정</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" t="str">
-        <x:v>AI 식단</x:v>
-      </x:c>
-      <x:c r="B35" t="str">
+      <x:c r="I42" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J42" s="61" t="str">
+        <x:v>전달 필드만 수정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="30" customHeight="1">
+      <x:c r="A43" s="72" t="str">
+        <x:v>생리 기록</x:v>
+      </x:c>
+      <x:c r="B43" s="77" t="str">
         <x:v>DELETE</x:v>
       </x:c>
-      <x:c r="C35" t="str">
-        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
-      </x:c>
-      <x:c r="D35" t="str">
-        <x:v>초안 음식 삭제</x:v>
-      </x:c>
-      <x:c r="E35" t="str">
+      <x:c r="C43" s="73" t="str">
+        <x:v>/api/v1/periods/{periodId}</x:v>
+      </x:c>
+      <x:c r="D43" s="73" t="str">
+        <x:v>생리 기간 삭제</x:v>
+      </x:c>
+      <x:c r="E43" s="73" t="str">
         <x:v>필요</x:v>
       </x:c>
-      <x:c r="F35" t="str">
+      <x:c r="F43" s="73" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="G35" t="str">
+      <x:c r="G43" s="73" t="str">
         <x:v>없음</x:v>
       </x:c>
-      <x:c r="H35" t="str">
+      <x:c r="H43" s="73" t="n">
         <x:v>204</x:v>
       </x:c>
-      <x:c r="I35" t="str">
-        <x:v>명세 확정</x:v>
-      </x:c>
-      <x:c r="J35"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" t="str">
-        <x:v>AI 식단</x:v>
-      </x:c>
-      <x:c r="B36" t="str">
+      <x:c r="I43" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J43" s="74"/>
+    </x:row>
+    <x:row r="44" ht="30" customHeight="1">
+      <x:c r="A44" s="59" t="str">
+        <x:v>마일리지</x:v>
+      </x:c>
+      <x:c r="B44" s="76" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C44" s="60" t="str">
+        <x:v>/api/v1/mileage</x:v>
+      </x:c>
+      <x:c r="D44" s="60" t="str">
+        <x:v>현재 잔액 조회</x:v>
+      </x:c>
+      <x:c r="E44" s="60" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F44" s="60" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G44" s="60" t="str">
+        <x:v>MileageBalanceResponse</x:v>
+      </x:c>
+      <x:c r="H44" s="60" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I44" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J44" s="61" t="str">
+        <x:v>일반 조회; 쓰기 잠금 없음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="30" customHeight="1">
+      <x:c r="A45" s="72" t="str">
+        <x:v>마일리지</x:v>
+      </x:c>
+      <x:c r="B45" s="77" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C45" s="73" t="str">
+        <x:v>/api/v1/mileage/history</x:v>
+      </x:c>
+      <x:c r="D45" s="73" t="str">
+        <x:v>마일리지 내역 조회</x:v>
+      </x:c>
+      <x:c r="E45" s="73" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F45" s="73" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G45" s="73" t="str">
+        <x:v>MileageHistoryResponse[]</x:v>
+      </x:c>
+      <x:c r="H45" s="73" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I45" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J45" s="74" t="str">
+        <x:v>최신순</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="30" customHeight="1">
+      <x:c r="A46" s="59" t="str">
+        <x:v>마일리지</x:v>
+      </x:c>
+      <x:c r="B46" s="76" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="C36" t="str">
-        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/record</x:v>
-      </x:c>
-      <x:c r="D36" t="str">
-        <x:v>초안을 일반 식단으로 기록</x:v>
-      </x:c>
-      <x:c r="E36" t="str">
+      <x:c r="C46" s="60" t="str">
+        <x:v>/api/v1/mileage/attendance</x:v>
+      </x:c>
+      <x:c r="D46" s="60" t="str">
+        <x:v>출석 보상 확인·지급</x:v>
+      </x:c>
+      <x:c r="E46" s="60" t="str">
         <x:v>필요</x:v>
       </x:c>
-      <x:c r="F36" t="str">
-        <x:v>Path: analysisId</x:v>
-      </x:c>
-      <x:c r="G36" t="str">
-        <x:v>MealResponse[]</x:v>
-      </x:c>
-      <x:c r="H36" t="str">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="I36" t="str">
-        <x:v>명세 확정</x:v>
-      </x:c>
-      <x:c r="J36" t="str">
-        <x:v>별도 확정 단계 없음</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" t="str">
-        <x:v>AI 식단</x:v>
-      </x:c>
-      <x:c r="B37" t="str">
-        <x:v>DELETE</x:v>
-      </x:c>
-      <x:c r="C37" t="str">
-        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}</x:v>
-      </x:c>
-      <x:c r="D37" t="str">
-        <x:v>분석 초안 취소</x:v>
-      </x:c>
-      <x:c r="E37" t="str">
+      <x:c r="F46" s="60" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G46" s="60" t="str">
+        <x:v>MileageRewardResponse</x:v>
+      </x:c>
+      <x:c r="H46" s="60" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I46" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J46" s="61" t="str">
+        <x:v>한국 시간 하루 1회</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="30" customHeight="1">
+      <x:c r="A47" s="72" t="str">
+        <x:v>마일리지</x:v>
+      </x:c>
+      <x:c r="B47" s="77" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C47" s="73" t="str">
+        <x:v>/api/v1/mileage/routine-streak/check</x:v>
+      </x:c>
+      <x:c r="D47" s="73" t="str">
+        <x:v>운동 연속 보상 확인·지급</x:v>
+      </x:c>
+      <x:c r="E47" s="73" t="str">
         <x:v>필요</x:v>
       </x:c>
-      <x:c r="F37" t="str">
+      <x:c r="F47" s="73" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="G37" t="str">
-        <x:v>없음</x:v>
-      </x:c>
-      <x:c r="H37" t="str">
-        <x:v>204</x:v>
-      </x:c>
-      <x:c r="I37" t="str">
-        <x:v>명세 확정</x:v>
-      </x:c>
-      <x:c r="J37" t="str">
-        <x:v>DRAFT는 7일 후 자동 삭제</x:v>
+      <x:c r="G47" s="73" t="str">
+        <x:v>MileageRewardResponse</x:v>
+      </x:c>
+      <x:c r="H47" s="73" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I47" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J47" s="74" t="str">
+        <x:v>지급 시 서버 쓰기 잠금</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="30" customHeight="1">
+      <x:c r="A48" s="59" t="str">
+        <x:v>AI 채팅</x:v>
+      </x:c>
+      <x:c r="B48" s="76" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C48" s="60" t="str">
+        <x:v>/api/v1/ai/chat</x:v>
+      </x:c>
+      <x:c r="D48" s="60" t="str">
+        <x:v>개인화 메시지 전송</x:v>
+      </x:c>
+      <x:c r="E48" s="60" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F48" s="60" t="str">
+        <x:v>AiChatRequest</x:v>
+      </x:c>
+      <x:c r="G48" s="60" t="str">
+        <x:v>AiChatResponse</x:v>
+      </x:c>
+      <x:c r="H48" s="60" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I48" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J48" s="61" t="str">
+        <x:v>최근 14일 기록 사용</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="30" customHeight="1">
+      <x:c r="A49" s="72" t="str">
+        <x:v>AI 채팅</x:v>
+      </x:c>
+      <x:c r="B49" s="77" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C49" s="73" t="str">
+        <x:v>/api/v1/ai/conversations</x:v>
+      </x:c>
+      <x:c r="D49" s="73" t="str">
+        <x:v>대화 목록 조회</x:v>
+      </x:c>
+      <x:c r="E49" s="73" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F49" s="73" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G49" s="73" t="str">
+        <x:v>AiConversationSummary[]</x:v>
+      </x:c>
+      <x:c r="H49" s="73" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I49" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J49" s="74" t="str">
+        <x:v>최신 대화순</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="30" customHeight="1">
+      <x:c r="A50" s="59" t="str">
+        <x:v>AI 채팅</x:v>
+      </x:c>
+      <x:c r="B50" s="76" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C50" s="60" t="str">
+        <x:v>/api/v1/ai/conversations/{conversationId}</x:v>
+      </x:c>
+      <x:c r="D50" s="60" t="str">
+        <x:v>대화 상세 조회</x:v>
+      </x:c>
+      <x:c r="E50" s="60" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F50" s="60" t="str">
+        <x:v>Path: conversationId</x:v>
+      </x:c>
+      <x:c r="G50" s="60" t="str">
+        <x:v>AiConversationDetail</x:v>
+      </x:c>
+      <x:c r="H50" s="60" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I50" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J50" s="61" t="str">
+        <x:v>완료 메시지만 반환</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="30" customHeight="1">
+      <x:c r="A51" s="72" t="str">
+        <x:v>AI 리포트</x:v>
+      </x:c>
+      <x:c r="B51" s="77" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C51" s="73" t="str">
+        <x:v>/api/v1/ai/reports</x:v>
+      </x:c>
+      <x:c r="D51" s="73" t="str">
+        <x:v>기간 리포트 생성</x:v>
+      </x:c>
+      <x:c r="E51" s="73" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F51" s="73" t="str">
+        <x:v>AiReportRequest</x:v>
+      </x:c>
+      <x:c r="G51" s="73" t="str">
+        <x:v>AiReportResponse</x:v>
+      </x:c>
+      <x:c r="H51" s="73" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I51" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J51" s="74" t="str">
+        <x:v>최대 31일</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="30" customHeight="1">
+      <x:c r="A52" s="59" t="str">
+        <x:v>AI 리포트</x:v>
+      </x:c>
+      <x:c r="B52" s="76" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C52" s="60" t="str">
+        <x:v>/api/v1/ai/reports/{reportId}</x:v>
+      </x:c>
+      <x:c r="D52" s="60" t="str">
+        <x:v>리포트 조회</x:v>
+      </x:c>
+      <x:c r="E52" s="60" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F52" s="60" t="str">
+        <x:v>Path: reportId</x:v>
+      </x:c>
+      <x:c r="G52" s="60" t="str">
+        <x:v>AiReportResponse</x:v>
+      </x:c>
+      <x:c r="H52" s="60" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I52" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J52" s="61"/>
+    </x:row>
+    <x:row r="53" ht="30" customHeight="1">
+      <x:c r="A53" s="72" t="str">
+        <x:v>AI 리포트</x:v>
+      </x:c>
+      <x:c r="B53" s="77" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C53" s="73" t="str">
+        <x:v>/api/v1/ai/reports/latest</x:v>
+      </x:c>
+      <x:c r="D53" s="73" t="str">
+        <x:v>최신 리포트 조회</x:v>
+      </x:c>
+      <x:c r="E53" s="73" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F53" s="73" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G53" s="73" t="str">
+        <x:v>AiReportResponse</x:v>
+      </x:c>
+      <x:c r="H53" s="73" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I53" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J53" s="74" t="str">
+        <x:v>없으면 404</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="30" customHeight="1">
+      <x:c r="A54" s="59" t="str">
+        <x:v>추천 식단</x:v>
+      </x:c>
+      <x:c r="B54" s="76" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C54" s="60" t="str">
+        <x:v>/api/v1/ai/meals/recommendations</x:v>
+      </x:c>
+      <x:c r="D54" s="60" t="str">
+        <x:v>최근 기록 기반 식단 추천</x:v>
+      </x:c>
+      <x:c r="E54" s="60" t="str">
+        <x:v>필요</x:v>
+      </x:c>
+      <x:c r="F54" s="60" t="str">
+        <x:v>MealRecommendationRequest</x:v>
+      </x:c>
+      <x:c r="G54" s="60" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="H54" s="60" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I54" s="63" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="J54" s="61" t="str">
+        <x:v>영양 미상은 null</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2343,7 +3119,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05e6edcc6e754597"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5aee7939fc0e406c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3626,13 +4402,59 @@
         <x:v>AI 식단</x:v>
       </x:c>
     </x:row>
+    <x:row r="56" ht="30" customHeight="1">
+      <x:c r="A56" s="59" t="str">
+        <x:v>MealRecommendationRequest</x:v>
+      </x:c>
+      <x:c r="B56" s="60" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="C56" s="60" t="str">
+        <x:v>date</x:v>
+      </x:c>
+      <x:c r="D56" s="60" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="E56" s="60" t="str">
+        <x:v>추천 대상일; YYYY-MM-DD</x:v>
+      </x:c>
+      <x:c r="F56" s="60" t="str">
+        <x:v>2026-08-19</x:v>
+      </x:c>
+      <x:c r="G56" s="61" t="str">
+        <x:v>추천 식단</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="30" customHeight="1">
+      <x:c r="A57" s="72" t="str">
+        <x:v>MealRecommendationRequest</x:v>
+      </x:c>
+      <x:c r="B57" s="73" t="str">
+        <x:v>mealType</x:v>
+      </x:c>
+      <x:c r="C57" s="73" t="str">
+        <x:v>enum</x:v>
+      </x:c>
+      <x:c r="D57" s="73" t="str">
+        <x:v>O</x:v>
+      </x:c>
+      <x:c r="E57" s="73" t="str">
+        <x:v>BREAKFAST/LUNCH/DINNER/SNACK</x:v>
+      </x:c>
+      <x:c r="F57" s="73" t="str">
+        <x:v>DINNER</x:v>
+      </x:c>
+      <x:c r="G57" s="74" t="str">
+        <x:v>추천 식단</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e06c40a28bc47cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4343958109a1447d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4445,13 +5267,237 @@
         <x:v>내부 신뢰도; 사용자에게 숫자 미표시</x:v>
       </x:c>
     </x:row>
+    <x:row r="58" ht="30" customHeight="1">
+      <x:c r="A58" s="59" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="B58" s="60" t="str">
+        <x:v>title</x:v>
+      </x:c>
+      <x:c r="C58" s="60" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D58" s="61" t="str">
+        <x:v>추천 식단 제목</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="30" customHeight="1">
+      <x:c r="A59" s="72" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="B59" s="73" t="str">
+        <x:v>description</x:v>
+      </x:c>
+      <x:c r="C59" s="73" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D59" s="74" t="str">
+        <x:v>식단 구성 설명</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="30" customHeight="1">
+      <x:c r="A60" s="59" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="B60" s="60" t="str">
+        <x:v>foods</x:v>
+      </x:c>
+      <x:c r="C60" s="60" t="str">
+        <x:v>RecommendedFoodItem[]</x:v>
+      </x:c>
+      <x:c r="D60" s="61" t="str">
+        <x:v>추천 음식 1~4개</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="30" customHeight="1">
+      <x:c r="A61" s="72" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="B61" s="73" t="str">
+        <x:v>totalKcal</x:v>
+      </x:c>
+      <x:c r="C61" s="73" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D61" s="74" t="str">
+        <x:v>음식별 값이 모두 있을 때의 서버 합계</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="30" customHeight="1">
+      <x:c r="A62" s="59" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="B62" s="60" t="str">
+        <x:v>totalCarbs</x:v>
+      </x:c>
+      <x:c r="C62" s="60" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D62" s="61" t="str">
+        <x:v>총 탄수화물 g; 일부 미상이면 null</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="30" customHeight="1">
+      <x:c r="A63" s="72" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="B63" s="73" t="str">
+        <x:v>totalProtein</x:v>
+      </x:c>
+      <x:c r="C63" s="73" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D63" s="74" t="str">
+        <x:v>총 단백질 g; 일부 미상이면 null</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="30" customHeight="1">
+      <x:c r="A64" s="59" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="B64" s="60" t="str">
+        <x:v>totalFat</x:v>
+      </x:c>
+      <x:c r="C64" s="60" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D64" s="61" t="str">
+        <x:v>총 지방 g; 일부 미상이면 null</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="30" customHeight="1">
+      <x:c r="A65" s="72" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="B65" s="73" t="str">
+        <x:v>reason</x:v>
+      </x:c>
+      <x:c r="C65" s="73" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D65" s="74" t="str">
+        <x:v>개인화 추천 이유</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="30" customHeight="1">
+      <x:c r="A66" s="59" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="B66" s="60" t="str">
+        <x:v>generatedAt</x:v>
+      </x:c>
+      <x:c r="C66" s="60" t="str">
+        <x:v>datetime</x:v>
+      </x:c>
+      <x:c r="D66" s="61" t="str">
+        <x:v>생성 시각(UTC ISO-8601)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="30" customHeight="1">
+      <x:c r="A67" s="72" t="str">
+        <x:v>RecommendedFoodItem</x:v>
+      </x:c>
+      <x:c r="B67" s="73" t="str">
+        <x:v>foodName</x:v>
+      </x:c>
+      <x:c r="C67" s="73" t="str">
+        <x:v>string</x:v>
+      </x:c>
+      <x:c r="D67" s="74" t="str">
+        <x:v>추천 음식명</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="30" customHeight="1">
+      <x:c r="A68" s="59" t="str">
+        <x:v>RecommendedFoodItem</x:v>
+      </x:c>
+      <x:c r="B68" s="60" t="str">
+        <x:v>amount</x:v>
+      </x:c>
+      <x:c r="C68" s="60" t="str">
+        <x:v>decimal|null</x:v>
+      </x:c>
+      <x:c r="D68" s="61" t="str">
+        <x:v>추정 양; 미상이면 null</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="30" customHeight="1">
+      <x:c r="A69" s="72" t="str">
+        <x:v>RecommendedFoodItem</x:v>
+      </x:c>
+      <x:c r="B69" s="73" t="str">
+        <x:v>amountUnit</x:v>
+      </x:c>
+      <x:c r="C69" s="73" t="str">
+        <x:v>string|null</x:v>
+      </x:c>
+      <x:c r="D69" s="74" t="str">
+        <x:v>양 단위; 미상이면 null</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="30" customHeight="1">
+      <x:c r="A70" s="59" t="str">
+        <x:v>RecommendedFoodItem</x:v>
+      </x:c>
+      <x:c r="B70" s="60" t="str">
+        <x:v>kcal</x:v>
+      </x:c>
+      <x:c r="C70" s="60" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D70" s="61" t="str">
+        <x:v>칼로리; 미상이면 null</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="30" customHeight="1">
+      <x:c r="A71" s="72" t="str">
+        <x:v>RecommendedFoodItem</x:v>
+      </x:c>
+      <x:c r="B71" s="73" t="str">
+        <x:v>carbs</x:v>
+      </x:c>
+      <x:c r="C71" s="73" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D71" s="74" t="str">
+        <x:v>탄수화물 g; 미상이면 null</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="30" customHeight="1">
+      <x:c r="A72" s="59" t="str">
+        <x:v>RecommendedFoodItem</x:v>
+      </x:c>
+      <x:c r="B72" s="60" t="str">
+        <x:v>protein</x:v>
+      </x:c>
+      <x:c r="C72" s="60" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D72" s="61" t="str">
+        <x:v>단백질 g; 미상이면 null</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="30" customHeight="1">
+      <x:c r="A73" s="72" t="str">
+        <x:v>RecommendedFoodItem</x:v>
+      </x:c>
+      <x:c r="B73" s="73" t="str">
+        <x:v>fat</x:v>
+      </x:c>
+      <x:c r="C73" s="73" t="str">
+        <x:v>integer|null</x:v>
+      </x:c>
+      <x:c r="D73" s="74" t="str">
+        <x:v>지방 g; 미상이면 null</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R620389ad3b9d4741"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f67a555875c4e04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5200,7 +6246,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf914ba74e6484577"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R384e7efed0dd47c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5453,13 +6499,41 @@
         <x:v>서버 내부 오류</x:v>
       </x:c>
     </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="59" t="str">
+        <x:v>AI_SERVICE_UNAVAILABLE</x:v>
+      </x:c>
+      <x:c r="B18" s="60" t="n">
+        <x:v>503</x:v>
+      </x:c>
+      <x:c r="C18" s="60" t="str">
+        <x:v>AI 기능을 준비 중입니다. 잠시 후 다시 시도해 주세요.</x:v>
+      </x:c>
+      <x:c r="D18" s="61" t="str">
+        <x:v>키 미설정 또는 제공자 호출 실패</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="72" t="str">
+        <x:v>AI_REPORT_NOT_FOUND</x:v>
+      </x:c>
+      <x:c r="B19" s="73" t="n">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="C19" s="73" t="str">
+        <x:v>AI 리포트를 찾을 수 없습니다.</x:v>
+      </x:c>
+      <x:c r="D19" s="74" t="str">
+        <x:v>사용자 리포트 없음</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c115b038bad43d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re73a47a5233f40d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5526,106 +6600,106 @@
         <x:v>결정 기준</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="33" t="str">
-        <x:v>AI 식단</x:v>
-      </x:c>
-      <x:c r="B4" s="33" t="str">
-        <x:v>사진/텍스트 multipart 형식</x:v>
-      </x:c>
-      <x:c r="C4" s="33" t="str">
-        <x:v>AI·프론트·백엔드</x:v>
-      </x:c>
-      <x:c r="D4" s="40" t="str">
-        <x:v>미확정</x:v>
-      </x:c>
-      <x:c r="E4" s="33" t="str">
-        <x:v>둘 중 최소 하나 필수</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="33" t="str">
-        <x:v>AI 식단</x:v>
-      </x:c>
-      <x:c r="B5" s="33" t="str">
-        <x:v>분석 응답 foods[] 및 DRAFT/CONFIRMED</x:v>
-      </x:c>
-      <x:c r="C5" s="33" t="str">
-        <x:v>AI·프론트·백엔드</x:v>
-      </x:c>
-      <x:c r="D5" s="40" t="str">
-        <x:v>미확정</x:v>
-      </x:c>
-      <x:c r="E5" s="33" t="str">
-        <x:v>사용자 수정 후 통계 반영</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="28" customHeight="1">
-      <x:c r="A6" s="33" t="str">
-        <x:v>AI 식단</x:v>
-      </x:c>
-      <x:c r="B6" s="33" t="str">
-        <x:v>파일 형식·최대 용량·요청 제한</x:v>
-      </x:c>
-      <x:c r="C6" s="33" t="str">
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="82" t="str">
+        <x:v>눈바디 AI</x:v>
+      </x:c>
+      <x:c r="B4" s="84" t="str">
+        <x:v>예상 변화 이미지 생성</x:v>
+      </x:c>
+      <x:c r="C4" s="84" t="str">
         <x:v>AI·백엔드</x:v>
       </x:c>
-      <x:c r="D6" s="40" t="str">
-        <x:v>미확정</x:v>
-      </x:c>
-      <x:c r="E6" s="33" t="str">
-        <x:v>JPG/PNG/HEIC 여부 포함</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="28" customHeight="1">
-      <x:c r="A7" s="33" t="str">
-        <x:v>눈바디</x:v>
-      </x:c>
-      <x:c r="B7" s="33" t="str">
-        <x:v>실제 이미지 저장소와 업로드 API</x:v>
-      </x:c>
-      <x:c r="C7" s="33" t="str">
+      <x:c r="D4" s="50" t="str">
+        <x:v>후순위</x:v>
+      </x:c>
+      <x:c r="E4" s="85" t="str">
+        <x:v>사진 기록과 추천 시술은 구현 완료</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="45" t="str">
+        <x:v>배포 AI</x:v>
+      </x:c>
+      <x:c r="B5" s="47" t="str">
+        <x:v>Railway OPENAI_API_KEY 등록</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>백엔드</x:v>
+      </x:c>
+      <x:c r="D5" s="50" t="str">
+        <x:v>필수 설정</x:v>
+      </x:c>
+      <x:c r="E5" s="48" t="str">
+        <x:v>미등록 시 모든 AI API가 503</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="A6" s="82" t="str">
+        <x:v>다이어리</x:v>
+      </x:c>
+      <x:c r="B6" s="84" t="str">
+        <x:v>기록 없음 응답 정책</x:v>
+      </x:c>
+      <x:c r="C6" s="84" t="str">
         <x:v>프론트·백엔드</x:v>
       </x:c>
-      <x:c r="D7" s="40" t="str">
-        <x:v>미확정</x:v>
-      </x:c>
-      <x:c r="E7" s="33" t="str">
-        <x:v>S3 등 결정 필요</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="33" t="str">
-        <x:v>눈바디 AI</x:v>
-      </x:c>
-      <x:c r="B8" s="33" t="str">
-        <x:v>예상 이미지 생성 요청/재시도</x:v>
-      </x:c>
-      <x:c r="C8" s="33" t="str">
-        <x:v>AI·백엔드</x:v>
-      </x:c>
-      <x:c r="D8" s="40" t="str">
-        <x:v>후순위</x:v>
-      </x:c>
-      <x:c r="E8" s="33" t="str">
-        <x:v>상태값은 정의 완료</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="28" customHeight="1">
-      <x:c r="A9" s="33" t="str">
-        <x:v>추천 시술</x:v>
-      </x:c>
-      <x:c r="B9" s="33" t="str">
-        <x:v>추천 필드·근거·정적 데이터 범위</x:v>
-      </x:c>
-      <x:c r="C9" s="33" t="str">
+      <x:c r="D6" s="50" t="str">
+        <x:v>현행 유지</x:v>
+      </x:c>
+      <x:c r="E6" s="85" t="str">
+        <x:v>현재 404 DIARY_NOT_FOUND; 프론트가 정상 처리</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="45" t="str">
+        <x:v>추천 식단</x:v>
+      </x:c>
+      <x:c r="B7" s="47" t="str">
+        <x:v>알레르기 정보 필드</x:v>
+      </x:c>
+      <x:c r="C7" s="47" t="str">
+        <x:v>기획·프론트·백엔드</x:v>
+      </x:c>
+      <x:c r="D7" s="50" t="str">
+        <x:v>추후</x:v>
+      </x:c>
+      <x:c r="E7" s="48" t="str">
+        <x:v>현재 정보가 없어 응답에서 확인 안내</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="82" t="str">
+        <x:v>스토어</x:v>
+      </x:c>
+      <x:c r="B8" s="84" t="str">
+        <x:v>구매 마일리지 지급 이벤트</x:v>
+      </x:c>
+      <x:c r="C8" s="84" t="str">
         <x:v>기획·백엔드</x:v>
       </x:c>
-      <x:c r="D9" s="40" t="str">
-        <x:v>미확정</x:v>
-      </x:c>
-      <x:c r="E9" s="33" t="str">
-        <x:v>예약·결제·실제 병원 연동 제외</x:v>
+      <x:c r="D8" s="50" t="str">
+        <x:v>MVP 제외</x:v>
+      </x:c>
+      <x:c r="E8" s="85" t="str">
+        <x:v>실제 주문 API 확정 후 연결</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="45" t="str">
+        <x:v>AI 운영</x:v>
+      </x:c>
+      <x:c r="B9" s="47" t="str">
+        <x:v>호출 제한·비용 모니터링</x:v>
+      </x:c>
+      <x:c r="C9" s="47" t="str">
+        <x:v>기획·백엔드</x:v>
+      </x:c>
+      <x:c r="D9" s="50" t="str">
+        <x:v>운영 전</x:v>
+      </x:c>
+      <x:c r="E9" s="48" t="str">
+        <x:v>MVP 일일 횟수 제한 없음</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5634,7 +6708,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cbe20c5d2564321"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raff8ce6145004f29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5741,352 +6815,468 @@
         <x:v>확정 여부</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="33" t="str">
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="82" t="str">
         <x:v>AI 식단</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="90" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="C4" s="33" t="str">
+      <x:c r="C4" s="84" t="str">
         <x:v>/api/v1/ai/nutrition/analyses</x:v>
       </x:c>
-      <x:c r="D4" s="33" t="str">
+      <x:c r="D4" s="84" t="str">
         <x:v>사진/텍스트 분석 및 DRAFT 생성</x:v>
       </x:c>
-      <x:c r="E4" s="33" t="str">
+      <x:c r="E4" s="84" t="str">
         <x:v>multipart</x:v>
       </x:c>
-      <x:c r="F4" s="33" t="str">
+      <x:c r="F4" s="84" t="str">
         <x:v>date,mealType,inputType,image 또는 text</x:v>
       </x:c>
-      <x:c r="G4" s="33" t="str">
+      <x:c r="G4" s="84" t="str">
         <x:v>NutritionAnalysisResponse</x:v>
       </x:c>
-      <x:c r="H4" s="33" t="str">
-        <x:v>PROCESSING/DRAFT</x:v>
-      </x:c>
-      <x:c r="I4" s="33" t="str">
+      <x:c r="H4" s="84" t="str">
+        <x:v>202/DRAFT</x:v>
+      </x:c>
+      <x:c r="I4" s="87" t="str">
         <x:v>확정</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="33" t="str">
+    <x:row r="5" ht="30" customHeight="1">
+      <x:c r="A5" s="45" t="str">
         <x:v>AI 식단</x:v>
       </x:c>
-      <x:c r="B5" s="37" t="str">
+      <x:c r="B5" s="75" t="str">
         <x:v>GET</x:v>
       </x:c>
-      <x:c r="C5" s="33" t="str">
+      <x:c r="C5" s="47" t="str">
         <x:v>/api/v1/ai/nutrition/analyses/{analysisId}</x:v>
       </x:c>
-      <x:c r="D5" s="33" t="str">
-        <x:v>분석 초안·진행 상태 조회</x:v>
-      </x:c>
-      <x:c r="E5" s="33" t="str">
+      <x:c r="D5" s="47" t="str">
+        <x:v>분석 초안·상태 조회</x:v>
+      </x:c>
+      <x:c r="E5" s="47" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="F5" s="33" t="str">
+      <x:c r="F5" s="47" t="str">
         <x:v>Path: analysisId</x:v>
       </x:c>
-      <x:c r="G5" s="33" t="str">
+      <x:c r="G5" s="47" t="str">
         <x:v>NutritionAnalysisResponse</x:v>
       </x:c>
-      <x:c r="H5" s="33" t="str">
-        <x:v>PROCESSING/DRAFT/FAILED</x:v>
-      </x:c>
-      <x:c r="I5" s="33" t="str">
+      <x:c r="H5" s="47" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I5" s="87" t="str">
         <x:v>확정</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="28" customHeight="1">
-      <x:c r="A6" s="33" t="str">
+    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="A6" s="82" t="str">
         <x:v>AI 식단</x:v>
       </x:c>
-      <x:c r="B6" s="37" t="str">
+      <x:c r="B6" s="90" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C6" s="84" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods</x:v>
+      </x:c>
+      <x:c r="D6" s="84" t="str">
+        <x:v>초안 음식 직접 추가</x:v>
+      </x:c>
+      <x:c r="E6" s="84" t="str">
+        <x:v>JSON</x:v>
+      </x:c>
+      <x:c r="F6" s="84" t="str">
+        <x:v>DraftFoodRequest</x:v>
+      </x:c>
+      <x:c r="G6" s="84" t="str">
+        <x:v>DraftFoodResponse</x:v>
+      </x:c>
+      <x:c r="H6" s="84" t="str">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="I6" s="87" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="45" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B7" s="75" t="str">
         <x:v>PATCH</x:v>
       </x:c>
-      <x:c r="C6" s="33" t="str">
+      <x:c r="C7" s="47" t="str">
         <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
       </x:c>
-      <x:c r="D6" s="33" t="str">
-        <x:v>AI 초안 음식 사용자 수정</x:v>
-      </x:c>
-      <x:c r="E6" s="33" t="str">
+      <x:c r="D7" s="47" t="str">
+        <x:v>초안 음식 부분 수정</x:v>
+      </x:c>
+      <x:c r="E7" s="47" t="str">
         <x:v>JSON</x:v>
       </x:c>
-      <x:c r="F6" s="33" t="str">
-        <x:v>foodName,amount,amountUnit,kcal,carbs,protein,fat</x:v>
-      </x:c>
-      <x:c r="G6" s="33" t="str">
+      <x:c r="F7" s="47" t="str">
+        <x:v>변경 필드</x:v>
+      </x:c>
+      <x:c r="G7" s="47" t="str">
         <x:v>DraftFoodResponse</x:v>
       </x:c>
-      <x:c r="H6" s="33" t="str">
-        <x:v>DRAFT</x:v>
-      </x:c>
-      <x:c r="I6" s="33" t="str">
+      <x:c r="H7" s="47" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I7" s="87" t="str">
         <x:v>확정</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="28" customHeight="1">
-      <x:c r="A7" s="33" t="str">
+    <x:row r="8" ht="30" customHeight="1">
+      <x:c r="A8" s="82" t="str">
         <x:v>AI 식단</x:v>
       </x:c>
-      <x:c r="B7" s="37" t="str">
+      <x:c r="B8" s="90" t="str">
+        <x:v>DELETE</x:v>
+      </x:c>
+      <x:c r="C8" s="84" t="str">
+        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
+      </x:c>
+      <x:c r="D8" s="84" t="str">
+        <x:v>초안 음식 삭제</x:v>
+      </x:c>
+      <x:c r="E8" s="84" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="F8" s="84" t="str">
+        <x:v>Path IDs</x:v>
+      </x:c>
+      <x:c r="G8" s="84" t="str">
+        <x:v>없음</x:v>
+      </x:c>
+      <x:c r="H8" s="84" t="str">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="I8" s="87" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="30" customHeight="1">
+      <x:c r="A9" s="45" t="str">
+        <x:v>AI 식단</x:v>
+      </x:c>
+      <x:c r="B9" s="75" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="C7" s="33" t="str">
+      <x:c r="C9" s="47" t="str">
         <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/record</x:v>
       </x:c>
-      <x:c r="D7" s="33" t="str">
-        <x:v>수정 여부와 관계없이 일반 식단으로 기록</x:v>
-      </x:c>
-      <x:c r="E7" s="33" t="str">
+      <x:c r="D9" s="47" t="str">
+        <x:v>일반 식단으로 기록</x:v>
+      </x:c>
+      <x:c r="E9" s="47" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="F7" s="33" t="str">
+      <x:c r="F9" s="47" t="str">
         <x:v>Path: analysisId</x:v>
       </x:c>
-      <x:c r="G7" s="33" t="str">
+      <x:c r="G9" s="47" t="str">
         <x:v>MealResponse[]</x:v>
       </x:c>
-      <x:c r="H7" s="33" t="str">
-        <x:v>RECORDED</x:v>
-      </x:c>
-      <x:c r="I7" s="33" t="str">
+      <x:c r="H9" s="47" t="str">
+        <x:v>201/RECORDED</x:v>
+      </x:c>
+      <x:c r="I9" s="87" t="str">
         <x:v>확정</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="33" t="str">
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="82" t="str">
         <x:v>AI 식단</x:v>
       </x:c>
-      <x:c r="B8" s="37" t="str">
+      <x:c r="B10" s="90" t="str">
         <x:v>DELETE</x:v>
       </x:c>
-      <x:c r="C8" s="33" t="str">
+      <x:c r="C10" s="84" t="str">
         <x:v>/api/v1/ai/nutrition/analyses/{analysisId}</x:v>
       </x:c>
-      <x:c r="D8" s="33" t="str">
+      <x:c r="D10" s="84" t="str">
         <x:v>분석 초안 취소</x:v>
       </x:c>
-      <x:c r="E8" s="33" t="str">
+      <x:c r="E10" s="84" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="F8" s="33" t="str">
+      <x:c r="F10" s="84" t="str">
         <x:v>Path: analysisId</x:v>
       </x:c>
-      <x:c r="G8" s="33" t="str">
+      <x:c r="G10" s="84" t="str">
         <x:v>없음</x:v>
       </x:c>
-      <x:c r="H8" s="33" t="str">
-        <x:v>CANCELLED</x:v>
-      </x:c>
-      <x:c r="I8" s="33" t="str">
+      <x:c r="H10" s="84" t="str">
+        <x:v>204/CANCELLED</x:v>
+      </x:c>
+      <x:c r="I10" s="87" t="str">
         <x:v>확정</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="28" customHeight="1">
-      <x:c r="A9" s="33" t="str">
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="45" t="str">
+        <x:v>추천 식단</x:v>
+      </x:c>
+      <x:c r="B11" s="75" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C11" s="47" t="str">
+        <x:v>/api/v1/ai/meals/recommendations</x:v>
+      </x:c>
+      <x:c r="D11" s="47" t="str">
+        <x:v>최근 14일·프로필 기반 추천</x:v>
+      </x:c>
+      <x:c r="E11" s="47" t="str">
+        <x:v>JSON</x:v>
+      </x:c>
+      <x:c r="F11" s="47" t="str">
+        <x:v>date,mealType</x:v>
+      </x:c>
+      <x:c r="G11" s="47" t="str">
+        <x:v>MealRecommendationResponse</x:v>
+      </x:c>
+      <x:c r="H11" s="47" t="str">
+        <x:v>200/503</x:v>
+      </x:c>
+      <x:c r="I11" s="87" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="82" t="str">
+        <x:v>AI 채팅</x:v>
+      </x:c>
+      <x:c r="B12" s="90" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C12" s="84" t="str">
+        <x:v>/api/v1/ai/chat</x:v>
+      </x:c>
+      <x:c r="D12" s="84" t="str">
+        <x:v>개인화 메시지 전송</x:v>
+      </x:c>
+      <x:c r="E12" s="84" t="str">
+        <x:v>JSON</x:v>
+      </x:c>
+      <x:c r="F12" s="84" t="str">
+        <x:v>conversationId?,message</x:v>
+      </x:c>
+      <x:c r="G12" s="84" t="str">
+        <x:v>AiChatResponse</x:v>
+      </x:c>
+      <x:c r="H12" s="84" t="str">
+        <x:v>200/503</x:v>
+      </x:c>
+      <x:c r="I12" s="87" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="45" t="str">
+        <x:v>AI 채팅</x:v>
+      </x:c>
+      <x:c r="B13" s="75" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C13" s="47" t="str">
+        <x:v>/api/v1/ai/conversations</x:v>
+      </x:c>
+      <x:c r="D13" s="47" t="str">
+        <x:v>대화 목록</x:v>
+      </x:c>
+      <x:c r="E13" s="47" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="F13" s="47" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G13" s="47" t="str">
+        <x:v>AiConversationSummary[]</x:v>
+      </x:c>
+      <x:c r="H13" s="47" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I13" s="87" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="59" t="str">
+        <x:v>AI 채팅</x:v>
+      </x:c>
+      <x:c r="B14" s="76" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C14" s="60" t="str">
+        <x:v>/api/v1/ai/conversations/{conversationId}</x:v>
+      </x:c>
+      <x:c r="D14" s="60" t="str">
+        <x:v>대화 상세</x:v>
+      </x:c>
+      <x:c r="E14" s="60" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="F14" s="60" t="str">
+        <x:v>Path: conversationId</x:v>
+      </x:c>
+      <x:c r="G14" s="60" t="str">
+        <x:v>AiConversationDetail</x:v>
+      </x:c>
+      <x:c r="H14" s="60" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I14" s="89" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="72" t="str">
+        <x:v>추천 시술</x:v>
+      </x:c>
+      <x:c r="B15" s="77" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C15" s="73" t="str">
+        <x:v>/api/v1/ai/procedures/recommendations</x:v>
+      </x:c>
+      <x:c r="D15" s="73" t="str">
+        <x:v>눈바디·프로필 기반 추천</x:v>
+      </x:c>
+      <x:c r="E15" s="73" t="str">
+        <x:v>JSON</x:v>
+      </x:c>
+      <x:c r="F15" s="73" t="str">
+        <x:v>bodyCheckId</x:v>
+      </x:c>
+      <x:c r="G15" s="73" t="str">
+        <x:v>ProcedureRecommendationsResponse</x:v>
+      </x:c>
+      <x:c r="H15" s="73" t="str">
+        <x:v>200/503</x:v>
+      </x:c>
+      <x:c r="I15" s="89" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="59" t="str">
+        <x:v>AI 리포트</x:v>
+      </x:c>
+      <x:c r="B16" s="76" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C16" s="60" t="str">
+        <x:v>/api/v1/ai/reports</x:v>
+      </x:c>
+      <x:c r="D16" s="60" t="str">
+        <x:v>기간 리포트 생성</x:v>
+      </x:c>
+      <x:c r="E16" s="60" t="str">
+        <x:v>JSON</x:v>
+      </x:c>
+      <x:c r="F16" s="60" t="str">
+        <x:v>from,to</x:v>
+      </x:c>
+      <x:c r="G16" s="60" t="str">
+        <x:v>AiReportResponse</x:v>
+      </x:c>
+      <x:c r="H16" s="60" t="str">
+        <x:v>200/503</x:v>
+      </x:c>
+      <x:c r="I16" s="89" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="72" t="str">
+        <x:v>AI 리포트</x:v>
+      </x:c>
+      <x:c r="B17" s="77" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C17" s="73" t="str">
+        <x:v>/api/v1/ai/reports/{reportId}</x:v>
+      </x:c>
+      <x:c r="D17" s="73" t="str">
+        <x:v>리포트 조회</x:v>
+      </x:c>
+      <x:c r="E17" s="73" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="F17" s="73" t="str">
+        <x:v>Path: reportId</x:v>
+      </x:c>
+      <x:c r="G17" s="73" t="str">
+        <x:v>AiReportResponse</x:v>
+      </x:c>
+      <x:c r="H17" s="73" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="I17" s="89" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="59" t="str">
+        <x:v>AI 리포트</x:v>
+      </x:c>
+      <x:c r="B18" s="76" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C18" s="60" t="str">
+        <x:v>/api/v1/ai/reports/latest</x:v>
+      </x:c>
+      <x:c r="D18" s="60" t="str">
+        <x:v>최신 리포트</x:v>
+      </x:c>
+      <x:c r="E18" s="60" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="F18" s="60" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="G18" s="60" t="str">
+        <x:v>AiReportResponse</x:v>
+      </x:c>
+      <x:c r="H18" s="60" t="str">
+        <x:v>200/404</x:v>
+      </x:c>
+      <x:c r="I18" s="89" t="str">
+        <x:v>확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="72" t="str">
         <x:v>눈바디 AI</x:v>
       </x:c>
-      <x:c r="B9" s="37" t="str">
+      <x:c r="B19" s="77" t="str">
         <x:v>POST</x:v>
       </x:c>
-      <x:c r="C9" s="33" t="str">
+      <x:c r="C19" s="73" t="str">
         <x:v>/api/v1/care/body-checks/{bodyCheckId}/analysis</x:v>
       </x:c>
-      <x:c r="D9" s="33" t="str">
-        <x:v>AI 예상 이미지 생성 요청</x:v>
-      </x:c>
-      <x:c r="E9" s="33" t="str">
-        <x:v>JSON/없음</x:v>
-      </x:c>
-      <x:c r="F9" s="33" t="str">
+      <x:c r="D19" s="73" t="str">
+        <x:v>예상 이미지 생성</x:v>
+      </x:c>
+      <x:c r="E19" s="73" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="F19" s="73" t="str">
         <x:v>Path: bodyCheckId</x:v>
       </x:c>
-      <x:c r="G9" s="33" t="str">
+      <x:c r="G19" s="73" t="str">
         <x:v>BodyCheckResponse</x:v>
       </x:c>
-      <x:c r="H9" s="33" t="str">
-        <x:v>ANALYZING</x:v>
-      </x:c>
-      <x:c r="I9" s="33" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="28" customHeight="1">
-      <x:c r="A10" s="33" t="str">
-        <x:v>AI 채팅</x:v>
-      </x:c>
-      <x:c r="B10" s="37" t="str">
-        <x:v>POST</x:v>
-      </x:c>
-      <x:c r="C10" s="33" t="str">
-        <x:v>/api/v1/ai/chat/sessions</x:v>
-      </x:c>
-      <x:c r="D10" s="33" t="str">
-        <x:v>대화 세션 생성</x:v>
-      </x:c>
-      <x:c r="E10" s="33" t="str">
-        <x:v>JSON</x:v>
-      </x:c>
-      <x:c r="F10" s="33" t="str">
-        <x:v>personaId?,characterId?</x:v>
-      </x:c>
-      <x:c r="G10" s="33" t="str">
-        <x:v>ChatSessionResponse</x:v>
-      </x:c>
-      <x:c r="H10" s="33" t="str">
-        <x:v>CREATED</x:v>
-      </x:c>
-      <x:c r="I10" s="33" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="28" customHeight="1">
-      <x:c r="A11" s="33" t="str">
-        <x:v>AI 채팅</x:v>
-      </x:c>
-      <x:c r="B11" s="37" t="str">
-        <x:v>POST</x:v>
-      </x:c>
-      <x:c r="C11" s="33" t="str">
-        <x:v>/api/v1/ai/chat/sessions/{sessionId}/messages</x:v>
-      </x:c>
-      <x:c r="D11" s="33" t="str">
-        <x:v>사용자 메시지 및 AI 응답</x:v>
-      </x:c>
-      <x:c r="E11" s="33" t="str">
-        <x:v>JSON</x:v>
-      </x:c>
-      <x:c r="F11" s="33" t="str">
-        <x:v>message</x:v>
-      </x:c>
-      <x:c r="G11" s="33" t="str">
-        <x:v>ChatMessageResponse</x:v>
-      </x:c>
-      <x:c r="H11" s="33" t="str">
-        <x:v>SUCCEEDED/FAILED</x:v>
-      </x:c>
-      <x:c r="I11" s="33" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="28" customHeight="1">
-      <x:c r="A12" s="33" t="str">
-        <x:v>AI 채팅</x:v>
-      </x:c>
-      <x:c r="B12" s="37" t="str">
-        <x:v>GET</x:v>
-      </x:c>
-      <x:c r="C12" s="33" t="str">
-        <x:v>/api/v1/ai/chat/sessions/{sessionId}/messages</x:v>
-      </x:c>
-      <x:c r="D12" s="33" t="str">
-        <x:v>대화 내역 조회</x:v>
-      </x:c>
-      <x:c r="E12" s="33" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="F12" s="33" t="str">
-        <x:v>Path: sessionId</x:v>
-      </x:c>
-      <x:c r="G12" s="33" t="str">
-        <x:v>ChatMessageResponse[]</x:v>
-      </x:c>
-      <x:c r="H12" s="33" t="str">
-        <x:v>200</x:v>
-      </x:c>
-      <x:c r="I12" s="33" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="28" customHeight="1">
-      <x:c r="A13" s="33" t="str">
-        <x:v>추천 시술</x:v>
-      </x:c>
-      <x:c r="B13" s="37" t="str">
-        <x:v>GET</x:v>
-      </x:c>
-      <x:c r="C13" s="33" t="str">
-        <x:v>/api/v1/procedures/recommendations</x:v>
-      </x:c>
-      <x:c r="D13" s="33" t="str">
-        <x:v>시술 추천 결과 조회</x:v>
-      </x:c>
-      <x:c r="E13" s="33" t="str">
-        <x:v>Query</x:v>
-      </x:c>
-      <x:c r="F13" s="33" t="str">
-        <x:v>bodyCheckId?</x:v>
-      </x:c>
-      <x:c r="G13" s="33" t="str">
-        <x:v>ProcedureRecommendation[]</x:v>
-      </x:c>
-      <x:c r="H13" s="33" t="str">
-        <x:v>200</x:v>
-      </x:c>
-      <x:c r="I13" s="33" t="str">
-        <x:v>초안</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>AI 식단</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>POST</x:v>
-      </x:c>
-      <x:c r="C14" t="str">
-        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods</x:v>
-      </x:c>
-      <x:c r="D14" t="str">
-        <x:v>초안 음식 직접 추가</x:v>
-      </x:c>
-      <x:c r="E14" t="str">
-        <x:v>JSON</x:v>
-      </x:c>
-      <x:c r="F14" t="str">
-        <x:v>DraftFoodRequest</x:v>
-      </x:c>
-      <x:c r="G14" t="str">
-        <x:v>DraftFoodResponse</x:v>
-      </x:c>
-      <x:c r="H14" t="str">
-        <x:v>DRAFT</x:v>
-      </x:c>
-      <x:c r="I14" t="str">
-        <x:v>확정</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>AI 식단</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>DELETE</x:v>
-      </x:c>
-      <x:c r="C15" t="str">
-        <x:v>/api/v1/ai/nutrition/analyses/{analysisId}/foods/{draftFoodId}</x:v>
-      </x:c>
-      <x:c r="D15" t="str">
-        <x:v>초안 음식 삭제</x:v>
-      </x:c>
-      <x:c r="E15" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="F15" t="str">
-        <x:v>Path: analysisId,draftFoodId</x:v>
-      </x:c>
-      <x:c r="G15" t="str">
-        <x:v>없음</x:v>
-      </x:c>
-      <x:c r="H15" t="str">
-        <x:v>DRAFT</x:v>
-      </x:c>
-      <x:c r="I15" t="str">
-        <x:v>확정</x:v>
+      <x:c r="H19" s="73" t="str">
+        <x:v>미구현</x:v>
+      </x:c>
+      <x:c r="I19" s="89" t="str">
+        <x:v>후순위</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6095,7 +7285,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1941aada9a214b10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fac83b71aa243ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6258,7 +7448,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae152ef940f24c0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf4ef93d0a014d43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>